<commit_message>
Add carousel-slider, columns-events blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- blocks/carousel-slider/carousel-slider.css
- blocks/columns-events/columns-events.css
- blocks/columns-events/columns-events.js
- tools/importer/import-homepage.bundle.js
- tools/importer/reports/en.report.json
- tools/importer/reports/import-homepage.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,13 +52,34 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-07-06T16:46:17.478Z</t>
+    <t>2026-07-13T13:54:12.111Z</t>
   </si>
   <si>
     <t>Homepage | Max-Planck-Gesellschaft</t>
   </si>
   <si>
     <t>https://www.mpg.de/en</t>
+  </si>
+  <si>
+    <t>26798800/democracy-cannot-be-taken-for-granted.report.json</t>
+  </si>
+  <si>
+    <t>["article-meta","article-aside","cards-news"]</t>
+  </si>
+  <si>
+    <t>26798800/democracy-cannot-be-taken-for-granted</t>
+  </si>
+  <si>
+    <t>article</t>
+  </si>
+  <si>
+    <t>2026-07-08T12:31:15.414Z</t>
+  </si>
+  <si>
+    <t>"Democracy cannot be taken for granted" | Max-Planck-Gesellschaft</t>
+  </si>
+  <si>
+    <t>https://www.mpg.de/26798800/democracy-cannot-be-taken-for-granted</t>
   </si>
 </sst>
 </file>
@@ -447,16 +468,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="36" customWidth="1"/>
-    <col min="8" max="8" width="23" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +528,32 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>